<commit_message>
Step 1: intake, dedupe, profile and exact-format readers
Email unpacked into attachments and content-bearing bodies. Byte-identical
files read once. Profile separates text-layer PDF pages from image pages.
UBL (PINT A-NZ) read as structure; XLSX, CSV, DOCX and email text read through
one grid representation with label-based header and table extraction.
Classifier reads the printed title and ignores field labels such as
'Purchase Order: PO-4105'. Gate met: csv, docx, eml body, ubl and xlsx all
100% on the synthetic pack.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y8XY8Vy9HYHXNVrttHXm8V
</commit_message>
<xml_diff>
--- a/corpus/synthetic/scenario_aug2026/GRN-7006.xlsx
+++ b/corpus/synthetic/scenario_aug2026/GRN-7006.xlsx
@@ -416,100 +416,107 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Goods Received Note</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>GRN-7006</t>
+          <t>Ridgeline Steel Fabrications Pty Ltd</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Goods Received Note</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Coastal Coatings Pty Ltd</t>
+          <t>GRN-7006</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PO Number</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PO-4106</t>
+          <t>Coastal Coatings Pty Ltd</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>PO Number</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PO-4106</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Received Date</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B5" s="1" t="n">
         <v>46253</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Item Code</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Qty Ordered</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Qty Received</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>UOM</t>
-        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Item Code</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Qty Ordered</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Qty Received</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>UOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>CC-ZP-20L</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Inorganic zinc primer 20L pail</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C8" t="n">
         <v>8</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>8</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>pail</t>
         </is>

</xml_diff>